<commit_message>
Close V2 foundations and global feedback phase
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,20 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R5ee0091ff85e40d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R6dcc6586b3e04481"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R26a159ebbe054cb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R410e026ec3334f57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R2804035048e14089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="6" r:id="R7056c1380e524f37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="7" r:id="R916ca4225e634ec8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="8" r:id="R3fca416263a84471"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="9" r:id="R1496c1bde13943ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="10" r:id="R60669496fa794d87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="11" r:id="R13aeedb693104a79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="12" r:id="R4290b17b19cd453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="13" r:id="R47997e518f84482c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="14" r:id="Rd4f330326bf84f97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R7a52594d2dc343f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="Rb4e62fdaab2b46dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Ra0b6a17594164eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R91cda96f266c4cb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rfdb6bf9b224b48d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R02ee73820c3c4fa3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R0a1bc7f6157c43ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Rd5dd53281fc24680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="9" r:id="R69431cc9b1ab4856"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="10" r:id="Rae4aa3ae6f90434f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="11" r:id="R5cc27ba95272479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="12" r:id="R5cf42d6d578b4915"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="13" r:id="Rd433b533009d43fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="14" r:id="Rf4040e7f2bb94c1a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="15" r:id="Reaa603ca6f1f4789"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="16" r:id="Rb90bdc64c53044bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -109,7 +111,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TenantAccessTable" displayName="TenantAccessTable" ref="A1:K5" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TenantAccessTable" displayName="TenantAccessTable" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -123,12 +125,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="FinanceTable" displayName="FinanceTable" ref="A1:K4" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="PlatformUXTable" displayName="PlatformUXTable" ref="A1:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -142,12 +144,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="AttachmentsTable" displayName="AttachmentsTable" ref="A1:K4" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="SalaryTable" displayName="SalaryTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -161,12 +163,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="CommunicationsTable" displayName="CommunicationsTable" ref="A1:K4" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="FinanceTable" displayName="FinanceTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -180,12 +182,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="PublicTrackingTable" displayName="PublicTrackingTable" ref="A1:K4" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="AttachmentsTable" displayName="AttachmentsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -199,12 +201,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="DeploymentSmokeTable" displayName="DeploymentSmokeTable" ref="A1:K4" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CommunicationsTable" displayName="CommunicationsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -218,12 +220,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RolesPermissionsTable" displayName="RolesPermissionsTable" ref="A1:K5" headerRowCount="1">
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="PublicTrackingTable" displayName="PublicTrackingTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -237,12 +239,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TenantIsolationTable" displayName="TenantIsolationTable" ref="A1:K5" headerRowCount="1">
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="DeploymentSmokeTable" displayName="DeploymentSmokeTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -256,12 +258,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CustomersTable" displayName="CustomersTable" ref="A1:K4" headerRowCount="1">
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="RolesPermissionsTable" displayName="RolesPermissionsTable" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -275,12 +277,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MeasurementsTable" displayName="MeasurementsTable" ref="A1:K4" headerRowCount="1">
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TenantIsolationTable" displayName="TenantIsolationTable" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -294,12 +296,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="OrdersTable" displayName="OrdersTable" ref="A1:K4" headerRowCount="1">
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CustomersTable" displayName="CustomersTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -313,12 +315,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="ProductionTable" displayName="ProductionTable" ref="A1:K4" headerRowCount="1">
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="MeasurementsTable" displayName="MeasurementsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -332,12 +334,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="AttendanceTable" displayName="AttendanceTable" ref="A1:K4" headerRowCount="1">
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -351,12 +353,12 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="SalaryTable" displayName="SalaryTable" ref="A1:K4" headerRowCount="1">
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="OrdersTable" displayName="OrdersTable" ref="A1:K6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -370,7 +372,45 @@
     <x:tableColumn id="10" name="Automation"/>
     <x:tableColumn id="11" name="Notes"/>
   </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ProductionTable" displayName="ProductionTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Test ID"/>
+    <x:tableColumn id="2" name="Priority"/>
+    <x:tableColumn id="3" name="Persona"/>
+    <x:tableColumn id="4" name="Tenant"/>
+    <x:tableColumn id="5" name="Preconditions"/>
+    <x:tableColumn id="6" name="Steps"/>
+    <x:tableColumn id="7" name="Expected Result"/>
+    <x:tableColumn id="8" name="Actual Result"/>
+    <x:tableColumn id="9" name="Status"/>
+    <x:tableColumn id="10" name="Automation"/>
+    <x:tableColumn id="11" name="Notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AttendanceTable" displayName="AttendanceTable" ref="A1:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Test ID"/>
+    <x:tableColumn id="2" name="Priority"/>
+    <x:tableColumn id="3" name="Persona"/>
+    <x:tableColumn id="4" name="Tenant"/>
+    <x:tableColumn id="5" name="Preconditions"/>
+    <x:tableColumn id="6" name="Steps"/>
+    <x:tableColumn id="7" name="Expected Result"/>
+    <x:tableColumn id="8" name="Actual Result"/>
+    <x:tableColumn id="9" name="Status"/>
+    <x:tableColumn id="10" name="Automation"/>
+    <x:tableColumn id="11" name="Notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -417,9 +457,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -432,12 +472,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -571,7 +657,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>TA-001</x:v>
       </x:c>
@@ -604,7 +690,7 @@
         <x:v>Use reachable email only after approval.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>TA-002</x:v>
       </x:c>
@@ -637,7 +723,7 @@
         <x:v>Disabled must never grant access.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>TA-003</x:v>
       </x:c>
@@ -670,7 +756,7 @@
         <x:v>Confirms account switching.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="31.5" customHeight="1">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>TA-004</x:v>
       </x:c>
@@ -706,7 +792,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7a91a698c8488f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb679e44de084c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -763,27 +849,27 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>FI-001</x:v>
+        <x:v>UX-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Any authorized user</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Expense category and payment mode exist.</x:v>
+        <x:v>A server mutation is available.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create expense.</x:v>
+        <x:v>Click its submit CTA.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Expense saves under selected tenant and appears in finance timeline.</x:v>
+        <x:v>The CTA immediately shows a spinner and action-specific pending label and is disabled until completion.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -794,72 +880,165 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>FI-002</x:v>
+        <x:v>UX-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Any authorized user</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Customer/order payments and salary payments exist.</x:v>
+        <x:v>A slow mutation is available.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open Finance overview.</x:v>
+        <x:v>Submit, then attempt another CTA, navigation, dialog close, Escape, and rapid resubmit.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Cash in/out, salary expense rollup, dues, and P&amp;L are consistent.</x:v>
+        <x:v>Conflicting interaction is blocked, focused pending dialogs cannot close, and only one mutation is accepted.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Manual UI</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>FI-003</x:v>
+        <x:v>UX-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Any authorized user</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Manager lacks finance permission.</x:v>
+        <x:v>An internal route link is available.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Attempt finance write action.</x:v>
+        <x:v>Click the link on desktop and mobile widths.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Action is denied.</x:v>
+        <x:v>A visible Opening page progress state appears and clears after navigation or the fail-safe timeout.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual UI</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
+    </x:row>
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>UX-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>A recoverable validation failure can be triggered in add-items or attendance import.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Submit invalid data.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Error feedback is visible, the draft remains available, and retry succeeds without duplicate submission.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str"/>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>UX-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Keyboard user</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Any shared dialog is available.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Open it, tab through controls, press Shift+Tab at the first control, close it, and repeat during a pending save.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Focus stays inside the modal, accessible name/description are exposed, focus returns to the trigger, and pending dialogs cannot close.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str"/>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>UX-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Boutique user</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Boutique-only tenant</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>The user has a role that would otherwise permit Tasks.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Open /tasks directly and attempt a Task server action.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>Both read and mutation paths reject access because Laundry is not enabled; Tasks remains hidden in navigation.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e8dea08a9e04c6e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26bd20c1fd9c46ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -916,58 +1095,58 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>AD-001</x:v>
+        <x:v>SA-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Customer exists.</x:v>
+        <x:v>Attendance and workers exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Upload JPG attachment on customer profile.</x:v>
+        <x:v>Create salary period and generate suggestions.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Attachment saves in private bucket and appears as thumbnail/gallery item.</x:v>
+        <x:v>Suggestions derive from tenant workers, attendance, work logs, and ledger only.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>AD-002</x:v>
+        <x:v>SA-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Tenant A and Tenant B</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Tenant B attachment ID known.</x:v>
+        <x:v>Existing active salary period.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open download URL from Tenant A session.</x:v>
+        <x:v>Create overlapping salary period.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>No signed URL is issued.</x:v>
+        <x:v>Action rejects overlap with clear message.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
@@ -978,27 +1157,27 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>AD-003</x:v>
+        <x:v>SA-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Customer-visible and internal attachments exist.</x:v>
+        <x:v>Salary calculation exists.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Open public tracking.</x:v>
+        <x:v>Finalize payable and record partial payment.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Internal/private attachments do not appear.</x:v>
+        <x:v>Final payable is preserved; salary_paid ledger entry appears in Finance rollup.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
@@ -1012,7 +1191,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R542e0ccd5eb249cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62b03e7fdbb4d08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1069,89 +1248,89 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>CO-001</x:v>
+        <x:v>FI-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Owner/Admin</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Settings access.</x:v>
+        <x:v>Expense category and payment mode exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create template with blocked variable such as {{worker_name}}.</x:v>
+        <x:v>Create expense.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Action rejects unsafe variable.</x:v>
+        <x:v>Expense saves under selected tenant and appears in finance timeline.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>CO-002</x:v>
+        <x:v>FI-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Order has customer phone/email.</x:v>
+        <x:v>Customer/order payments and salary payments exist.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Queue manual tracking link dry-run.</x:v>
+        <x:v>Open Finance overview.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Message queue and log are tenant-scoped and marked dry-run.</x:v>
+        <x:v>Cash in/out, salary expense rollup, dues, and P&amp;L are consistent.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>CO-003</x:v>
+        <x:v>FI-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Owner/Admin</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Communication channel settings open.</x:v>
+        <x:v>Manager lacks finance permission.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Attempt to set live mode.</x:v>
+        <x:v>Attempt finance write action.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Action rejects live sending in MVP slice.</x:v>
+        <x:v>Action is denied.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
@@ -1165,7 +1344,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dbdef987d1a44fe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15c8f2b8a88a4851"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1222,58 +1401,58 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>PT-001</x:v>
+        <x:v>AD-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Valid tracking token exists.</x:v>
+        <x:v>Customer exists.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Open /track/[token].</x:v>
+        <x:v>Upload JPG attachment on customer profile.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Page loads without Clerk and shows tenant branding, order dates, item names, and customer-safe statuses.</x:v>
+        <x:v>Attachment saves in private bucket and appears as thumbnail/gallery item.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>PT-002</x:v>
+        <x:v>AD-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Invalid/random token.</x:v>
+        <x:v>Tenant B attachment ID known.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open /track/random-token.</x:v>
+        <x:v>Open download URL from Tenant A session.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Page returns not found.</x:v>
+        <x:v>No signed URL is issued.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
@@ -1284,9 +1463,9 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>PT-003</x:v>
+        <x:v>AD-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P0</x:v>
@@ -1298,13 +1477,13 @@
         <x:v>Public</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Order has measurements, workers, stage names, notes, salary, private attachments.</x:v>
+        <x:v>Customer-visible and internal attachments exist.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Open tracking token.</x:v>
+        <x:v>Open public tracking.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>None of those internal fields appear in payload or UI.</x:v>
+        <x:v>Internal/private attachments do not appear.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
@@ -1313,14 +1492,12 @@
       <x:c r="J4" s="6" t="str">
         <x:v>Manual + Automated</x:v>
       </x:c>
-      <x:c r="K4" s="6" t="str">
-        <x:v>Regression for 2026-06-04 hardening patch.</x:v>
-      </x:c>
+      <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92cb84c2e1ac4808"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da8bfdbee634abe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1377,9 +1554,9 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>DS-001</x:v>
+        <x:v>CO-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P0</x:v>
@@ -1388,92 +1565,400 @@
         <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>Preview</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Preview deployment and env vars configured.</x:v>
+        <x:v>Settings access.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Open sign-in, selector, dashboard, orders, customers, production, finance.</x:v>
+        <x:v>Create template with blocked variable such as {{worker_name}}.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>All routes return 200 for authorized user.</x:v>
+        <x:v>Action rejects unsafe variable.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>DS-002</x:v>
+        <x:v>CO-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>System</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Preview</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Migrations applied.</x:v>
+        <x:v>Order has customer phone/email.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Run typecheck, lint, and production build.</x:v>
+        <x:v>Queue manual tracking link dry-run.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>All commands pass.</x:v>
+        <x:v>Message queue and log are tenant-scoped and marked dry-run.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>DS-003</x:v>
+        <x:v>CO-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
         <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Clean boutique tenant</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Fresh pilot tenant exists.</x:v>
+        <x:v>Communication channel settings open.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Run one order from setup through tracking and dry-run communication.</x:v>
+        <x:v>Attempt to set live mode.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Pilot loop completes without cross-tenant leakage or role surprises.</x:v>
+        <x:v>Action rejects live sending in MVP slice.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5651a4e578e942d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bee6813454441d3"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Test ID</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Persona</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>Tenant</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>Preconditions</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Steps</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Actual Result</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="J1" s="4" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="K1" s="4" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>PT-001</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>Public customer</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>Public</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>Valid tracking token exists.</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>Open /track/[token].</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str">
+        <x:v>Page loads without Clerk and shows tenant branding, order dates, item names, and customer-safe statuses.</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="str"/>
+      <x:c r="I2" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K2" s="6" t="str"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>PT-002</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>Public customer</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>Public</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>Invalid/random token.</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>Open /track/random-token.</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>Page returns not found.</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="str"/>
+      <x:c r="I3" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str"/>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>PT-003</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>Public customer</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>Public</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Order has measurements, workers, stage names, notes, salary, private attachments.</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Open tracking token.</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>None of those internal fields appear in payload or UI.</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str"/>
+      <x:c r="I4" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str">
+        <x:v>Regression for 2026-06-04 hardening patch.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R763ccde7df724c90"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Test ID</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Persona</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>Tenant</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>Preconditions</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Steps</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Actual Result</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="J1" s="4" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="K1" s="4" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>DS-001</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>Preview</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>Preview deployment and env vars configured.</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>Open sign-in, selector, dashboard, orders, customers, production, finance.</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str">
+        <x:v>All routes return 200 for authorized user.</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="str"/>
+      <x:c r="I2" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="K2" s="6" t="str"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>DS-002</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>Preview</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>Migrations applied.</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>Run typecheck, lint, and production build.</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>All commands pass.</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="str"/>
+      <x:c r="I3" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str"/>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>DS-003</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>Clean boutique tenant</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Fresh pilot tenant exists.</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Run one order from setup through tracking and dry-run communication.</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>Pilot loop completes without cross-tenant leakage or role surprises.</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str"/>
+      <x:c r="I4" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>Manual</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91f48216b290431c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1530,7 +2015,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>RP-001</x:v>
       </x:c>
@@ -1561,7 +2046,7 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>RP-002</x:v>
       </x:c>
@@ -1592,7 +2077,7 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>RP-003</x:v>
       </x:c>
@@ -1623,7 +2108,7 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
-    <x:row r="5" ht="31.5" customHeight="1">
+    <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>RP-004</x:v>
       </x:c>
@@ -1657,7 +2142,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdefa176a3532431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R028e3ca4a91d4d22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1714,7 +2199,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>TI-001</x:v>
       </x:c>
@@ -1747,7 +2232,7 @@
         <x:v>Cover ID-based pages.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>TI-002</x:v>
       </x:c>
@@ -1780,7 +2265,7 @@
         <x:v>Private storage path must remain hidden.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>TI-003</x:v>
       </x:c>
@@ -1811,7 +2296,7 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
-    <x:row r="5" ht="31.5" customHeight="1">
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>TI-004</x:v>
       </x:c>
@@ -1847,7 +2332,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45e5965bcf5b4ee1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9083ce6a49ec4d39"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1904,7 +2389,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>CU-001</x:v>
       </x:c>
@@ -1935,12 +2420,12 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>CU-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
         <x:v>Manager</x:v>
@@ -1949,24 +2434,26 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Existing customer has phone.</x:v>
+        <x:v>An active customer already has a mobile number.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Create another customer with similar phone.</x:v>
+        <x:v>Attempt to create another customer using the same normalized Indian mobile in 10-digit, leading 0, +91, or 0091 form.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Suggestions appear, but duplicate creation remains allowed.</x:v>
+        <x:v>Server blocks the duplicate, resolves the existing customer, and the inline order flow selects that customer without losing the order draft.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual</x:v>
-      </x:c>
-      <x:c r="K3" s="6" t="str"/>
-    </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str">
+        <x:v>Application-level normalized mobile guard; mobile remains optional.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>CU-003</x:v>
       </x:c>
@@ -2000,7 +2487,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf65cb07c5329456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra24be0598322420c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2057,7 +2544,7 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>ME-001</x:v>
       </x:c>
@@ -2088,7 +2575,7 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>ME-002</x:v>
       </x:c>
@@ -2119,7 +2606,7 @@
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>ME-003</x:v>
       </x:c>
@@ -2153,7 +2640,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd2c301c83634db5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf330602bce4b4ed6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2210,27 +2697,27 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>OR-001</x:v>
+        <x:v>CF-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Customer, item type, workflow, payment mode exist.</x:v>
+        <x:v>Item types, stages, statuses, workgroups, payment modes, and expense categories exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create order with two items and partial payment.</x:v>
+        <x:v>Edit each master and toggle an active state.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Order number auto-generates; items and payment save under selected tenant.</x:v>
+        <x:v>Each tenant-owned record updates; historical production and finance references remain intact.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -2241,72 +2728,196 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>OR-002</x:v>
+        <x:v>CF-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Order exists.</x:v>
+        <x:v>Tenant B configuration IDs are known.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Edit item notes, due date, delivery override, and fit reference.</x:v>
+        <x:v>Submit Tenant B IDs from Tenant A edit forms.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Allowed fields update; destructive changes are not exposed.</x:v>
+        <x:v>Every action rejects or returns not found; no Tenant B record changes.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>OR-003</x:v>
+        <x:v>CF-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Tenant A and Tenant B</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Known Tenant B order ID.</x:v>
+        <x:v>Worker, workflow, locations, teams, measurement fields, standard sizes, and customer measurements exist.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Open Tenant B order ID from Tenant A session.</x:v>
+        <x:v>Edit each record, replace a workflow stage sequence, repeat with an inactive/foreign stage, then simultaneously activate an inactive workflow while deactivating its sole active stage.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Order detail returns not found or blocked.</x:v>
+        <x:v>Valid changes save with tenant/reference validation; workflow create/default/stage writes are atomic; invalid replacement leaves the prior sequence intact; workflow-then-stage locking allows exactly one conflicting state change to commit; existing history remains available.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Database + Manual + Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
+    </x:row>
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>CF-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>An order payment exists.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Open Finance payment correction, change allowed fields, enter a reason, and save.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>One order-locking transaction updates the payment and summary and stores immutable old/new values, actor, and reason without deleting payment history.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Database + Manual</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str"/>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>CF-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>All tenants</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Expense-default migration is ready and tenants contain custom or partial categories.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Apply migration, inspect existing tenants, then create a fresh tenant.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Each tenant has the ten defaults exactly once by normalized name; custom, renamed, inactive, and deleted history is not overwritten or revived.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str"/>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>CF-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>An order has an outstanding balance.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Submit two concurrent payments whose combined value exceeds the balance.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>The order lock serializes both requests; at most one succeeds and payment rows never exceed the order total.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str"/>
+    </x:row>
+    <x:row r="8" ht="66" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>CF-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>Measurement fields, sizes, measurements, and order history exist.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Try to change a field key/item type or reassign any existing size/measurement to another item type.</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Creation identities are always immutable while labels, dimensions, notes, order, and active state remain editable; concurrent order creation cannot create an incompatible reference.</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R93eb9353625542f1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43ce480267644eb9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2363,9 +2974,9 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>PR-001</x:v>
+        <x:v>OR-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P0</x:v>
@@ -2377,13 +2988,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Order item has workflow instance and ready stage.</x:v>
+        <x:v>Customer, item type, workflow, payment mode exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Start stage with allowed worker.</x:v>
+        <x:v>Create order with two items and partial payment.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Stage starts, work log is created, item history records event.</x:v>
+        <x:v>Order number auto-generates; items and payment save under selected tenant.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -2394,12 +3005,12 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>PR-002</x:v>
+        <x:v>OR-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
         <x:v>Manager</x:v>
@@ -2408,58 +3019,124 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Worker outside allowed workgroup exists.</x:v>
+        <x:v>Order exists.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Attempt to start stage with disallowed worker.</x:v>
+        <x:v>Edit item notes, due date, delivery override, and fit reference.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Action rejects worker assignment.</x:v>
+        <x:v>Allowed fields update; destructive changes are not exposed.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>PR-003</x:v>
+        <x:v>OR-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
         <x:v>Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>In-progress stage exists.</x:v>
+        <x:v>Known Tenant B order ID.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Complete stage.</x:v>
+        <x:v>Open Tenant B order ID from Tenant A session.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Current stage completes and next stage becomes ready when applicable.</x:v>
+        <x:v>Order detail returns not found or blocked.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str"/>
+    </x:row>
+    <x:row r="5" ht="92.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>OR-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>An active legacy Boutique order exists with payment history; active item types and workflows are configured.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Open order detail, add two new item rows in one save, and use a customer measurement on one row and a standard size on the other.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Both items save atomically, each gets its own workflow instance and first ready stage, item history records the addition, totals recalculate from all active items, payments remain unchanged, and production/finance/public tracking refresh.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
         <x:v>Manual + Automated</x:v>
       </x:c>
-      <x:c r="K4" s="6" t="str"/>
+      <x:c r="K5" s="6" t="str">
+        <x:v>Run against an unpaid or paid order; a paid order can become partially paid after the total increases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>OR-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Tenant A and Tenant B</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>An editable Tenant A order exists; Tenant B IDs and an incompatible measurement or size are known.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Attempt a multi-row add with one invalid or foreign reference, retry the same valid request key, and attempt rapid duplicate submission.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Invalid batches roll back completely; tenant and fit-reference mismatches are rejected; an idempotent retry returns the original result; the pending dialog blocks edits, closing, and duplicate submission while preserving rows on error.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Automated + Manual UI</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str">
+        <x:v>Also confirm cancelled and fully delivered orders cannot add items.</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ba6c0ec9fc34702"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf054fa3a54e346b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2516,12 +3193,12 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>AT-001</x:v>
+        <x:v>PR-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
         <x:v>Manager</x:v>
@@ -2530,13 +3207,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Active workers exist.</x:v>
+        <x:v>Order item has workflow instance and ready stage.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Mark daily attendance and save sheet.</x:v>
+        <x:v>Start stage with allowed worker.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>One tenant-scoped attendance row per marked worker/date is saved.</x:v>
+        <x:v>Stage starts, work log is created, item history records event.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -2547,12 +3224,12 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>AT-002</x:v>
+        <x:v>PR-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
         <x:v>Manager</x:v>
@@ -2561,58 +3238,58 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Attendance data exists.</x:v>
+        <x:v>Worker outside allowed workgroup exists.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open overview with 14-day range and worker filters.</x:v>
+        <x:v>Attempt to start stage with disallowed worker.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Charts, regularity, and attention board reflect selected workers only.</x:v>
+        <x:v>Action rejects worker assignment.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>AT-003</x:v>
+        <x:v>PR-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
         <x:v>Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Tenant A and Tenant B</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Tenant B worker ID known.</x:v>
+        <x:v>In-progress stage exists.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Submit attendance for Tenant B worker ID from Tenant A.</x:v>
+        <x:v>Complete stage.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Action rejects worker ownership mismatch.</x:v>
+        <x:v>Current stage completes and next stage becomes ready when applicable.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6dd90da2c90c41bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cbf1a490d9e4687"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2669,27 +3346,27 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>SA-001</x:v>
+        <x:v>AT-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Attendance and workers exist.</x:v>
+        <x:v>Active workers exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create salary period and generate suggestions.</x:v>
+        <x:v>Mark daily attendance and save sheet.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Suggestions derive from tenant workers, attendance, work logs, and ledger only.</x:v>
+        <x:v>One tenant-scoped attendance row per marked worker/date is saved.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -2700,72 +3377,355 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="31.5" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>SA-002</x:v>
+        <x:v>AT-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Existing active salary period.</x:v>
+        <x:v>Attendance data exists.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Create overlapping salary period.</x:v>
+        <x:v>Open overview with 14-day range and worker filters.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Action rejects overlap with clear message.</x:v>
+        <x:v>Charts, regularity, and attention board reflect selected workers only.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="31.5" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>SA-003</x:v>
+        <x:v>AT-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Salary calculation exists.</x:v>
+        <x:v>Tenant B worker ID known.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Finalize payable and record partial payment.</x:v>
+        <x:v>Submit attendance for Tenant B worker ID from Tenant A.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Final payable is preserved; salary_paid ledger entry appears in Finance rollup.</x:v>
+        <x:v>Action rejects worker ownership mismatch.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str"/>
+    </x:row>
+    <x:row r="5" ht="66" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>AT-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>The supplied sample .xls report is available and some active worker profile names match exactly after normalization.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Upload the report and preview it.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Preview writes nothing and shows report month, exact matches, unmatched/ambiguous workers, new/update rows, future dates, blank statuses, and unknown statuses.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
         <x:v>Manual + Automated</x:v>
       </x:c>
-      <x:c r="K4" s="6" t="str"/>
+      <x:c r="K5" s="6" t="str">
+        <x:v>Use docs_v2/sample_Attendance_Report.xls.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>AT-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Preview contains matched and unmatched source workers.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Confirm import.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Only exact normalized active-worker matches are inserted or updated; no worker profiles are created and skipped names remain unchanged.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str">
+        <x:v>No fuzzy matching.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>AT-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Tenant A and Tenant B</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>Both tenants contain workers; a workbook name matches only Tenant B.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Import while selected into Tenant A.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>Tenant B worker and attendance rows are untouched; the source worker is skipped for Tenant A.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str"/>
+    </x:row>
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>AT-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>A worker/date already has manual attendance and a note.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Preview and confirm a workbook containing that worker/date.</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Preview labels the row as an update; status/time/hours update atomically and the existing free-text note is preserved.</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str"/>
+    </x:row>
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>AT-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>A valid preview and idempotency key exist.</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Confirm twice or rapidly double-click confirmation.</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>The second request returns the stored receipt and creates no duplicate attendance or import receipt.</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>Database + Manual UI</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str"/>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>AT-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>A workbook contains a future date, blank status, unknown status, and duplicate normalized worker name.</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Preview and confirm.</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>Those rows/workers are explicitly reported and skipped; valid exact matches still import.</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str"/>
+      <x:c r="I10" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="str"/>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>AT-010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>A confirmed batch contains a tampered/invalid referenced row.</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Execute confirmation through the database contract.</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>The complete transaction rolls back and no partial attendance/import receipt remains.</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str"/>
+      <x:c r="I11" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str"/>
+    </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>AT-011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>A confirmed attendance import receipt exists.</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Attempt direct update and direct delete as service role, then delete its parent test tenant through approved cleanup.</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>Direct mutation is rejected as immutable; approved parent cascade cleanup remains possible.</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str"/>
+    </x:row>
+    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>AT-012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>Adversarial .xlsx fixtures contain oversized expansion, unsafe ratios, local/central header mismatches, renamed extensions, or excessive entries/sheets/rows/columns/cells.</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Preview each fixture.</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>Every unsafe workbook is rejected before worksheet materialization via signature/header checks and hard-capped inflation; no receipt is written; valid .xls and .xlsx structures still reach format validation.</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str"/>
+      <x:c r="I13" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re3bdc91054e44e91"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15aa678c65ba4af0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add tenant-safe customer file import
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,22 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R7a52594d2dc343f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="Rb4e62fdaab2b46dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Ra0b6a17594164eef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R91cda96f266c4cb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rfdb6bf9b224b48d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R02ee73820c3c4fa3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R0a1bc7f6157c43ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Rd5dd53281fc24680"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="9" r:id="R69431cc9b1ab4856"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="10" r:id="Rae4aa3ae6f90434f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="11" r:id="R5cc27ba95272479d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="12" r:id="R5cf42d6d578b4915"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="13" r:id="Rd433b533009d43fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="14" r:id="Rf4040e7f2bb94c1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="15" r:id="Reaa603ca6f1f4789"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="16" r:id="Rb90bdc64c53044bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R9bfb1b62831542d5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R3d9852b677d34f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R0ea01a1294064246"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R31a22ee6d5894255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R2123f9bb2b9148bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R5a2e34ada3894e9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R7ec4d38a3cc04c8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Ra7f89356bdd64280"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="9" r:id="Rb09e4cec17574a0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="10" r:id="Re65e3417f55a46b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="11" r:id="R99bc6cb0b325496f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="12" r:id="R76a2d76a3bba4140"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="13" r:id="R4cdeab9e99794792"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="14" r:id="R86bea42466244a76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="15" r:id="Rd7b14aeecf114b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="16" r:id="R07e98f6ad000437c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,7 +301,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CustomersTable" displayName="CustomersTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="CustomersTable" displayName="CustomersTable" ref="A1:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -792,7 +792,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb679e44de084c86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2c0d4684df4017"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1038,7 +1038,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26bd20c1fd9c46ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca95ffcf2e164898"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1191,7 +1191,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re62b03e7fdbb4d08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reacbea6ca5874ce7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1344,7 +1344,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15c8f2b8a88a4851"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfab3561be0af45a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1497,7 +1497,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da8bfdbee634abe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e4aef33dc6a43fb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1650,7 +1650,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bee6813454441d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4e0a11e67304145"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1805,7 +1805,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R763ccde7df724c90"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebb6f3d01ac242ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1958,7 +1958,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R91f48216b290431c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcca074f367cf46c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2142,7 +2142,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R028e3ca4a91d4d22"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0456c6f809314073"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2332,7 +2332,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9083ce6a49ec4d39"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a04a024ae7a4b83"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2484,10 +2484,142 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
+    <x:row r="5" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>CU-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>CSV and XLSX customer fixtures contain valid Indian, explicit international, country-assisted foreign, ambiguous foreign, blank-name, malformed, and over-limit cases.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Preview each file, including files larger than 5 MB or 5,000 data rows.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Valid rows preview without writes; foreign numbers normalize only with explicit/country context; ambiguous phones, blank names, malformed files, and limits are rejected or counted; the invalid/skipped count is visible.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Automated + Manual</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str">
+        <x:v>Manager and other roles must not see or execute import.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>CU-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Tenant contains matching Shopify IDs, normalized phones, exact emails, blank fields, and conflicting populated fields.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Preview rows covering every matching path and resolve each email-only row as reuse, create separate, or skip.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Shopify ID wins, then normalized phone; cross-key disagreement is invalid; phone matches always reuse; email-only matches wait for an explicit decision; blank fields can be filled and populated conflicts remain unchanged and visible.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Automated + Manual</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str">
+        <x:v>No email address is used as a fake customer name.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>CU-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Tenant A and Tenant B</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>A valid approved preview, foreign tenant IDs, and one intentionally invalid row are available.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Confirm the batch, retry the same idempotency key, attempt a tampered/foreign target, and force one row failure.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>The valid batch commits once; retry returns the receipt; tenant/tampered rows are rejected; any failure rolls back customers, addresses, identities, metadata, and receipt with no partial import.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str">
+        <x:v>Database function is service-role-only and revalidates every target.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>CU-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>Rows contain complete/incomplete addresses and Shopify totals, order counts, tags, tax and marketing flags.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Confirm import, inspect customer/address records, reports, finance, and messaging configuration.</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Complete addresses become structured defaults only when no default exists; incomplete text remains legacy data; metadata is retained read-only; no historical orders/finance entries, report totals, or messaging consent are created.</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Database + Manual</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str">
+        <x:v>Metadata is a future Shopify-integration foundation only.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra24be0598322420c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c6bf608d1f74036"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2640,7 +2772,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf330602bce4b4ed6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb47fb2262b44fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2917,7 +3049,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43ce480267644eb9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae819d272e534ccd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3136,7 +3268,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf054fa3a54e346b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22b3cf844f3a416e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3289,7 +3421,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cbf1a490d9e4687"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R248fd2e4adae4e6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3725,7 +3857,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15aa678c65ba4af0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R889b1657e31743e5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add stage worker contributions and analytics
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,22 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R9bfb1b62831542d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R3d9852b677d34f61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R0ea01a1294064246"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R31a22ee6d5894255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R2123f9bb2b9148bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R5a2e34ada3894e9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R7ec4d38a3cc04c8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Ra7f89356bdd64280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="9" r:id="Rb09e4cec17574a0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="10" r:id="Re65e3417f55a46b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="11" r:id="R99bc6cb0b325496f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="12" r:id="R76a2d76a3bba4140"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="13" r:id="R4cdeab9e99794792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="14" r:id="R86bea42466244a76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="15" r:id="Rd7b14aeecf114b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="16" r:id="R07e98f6ad000437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R96ad21cb61d546eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R82c4f6f4e1f14435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R9a62a31d409f4068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R20690d98c3624970"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R09ff56c615c347cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R6ade54b371b04a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R4d3c4cda2b0b4554"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="R9014ec8c76194146"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="R981c764b9baa48ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="R9129b09c68c54a42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="Rf595399044964d03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="Rb7359c886cd84684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="Rc313f18d089f4ac6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="Rae0df2c18cab4997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R947e1a403ad0437b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R04cfb3c9642c4ec7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R7e8639b1f2684183"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -130,7 +131,7 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="PlatformUXTable" displayName="PlatformUXTable" ref="A1:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="AttendanceTable" displayName="AttendanceTable" ref="A1:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -149,7 +150,7 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="SalaryTable" displayName="SalaryTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="PlatformUXTable" displayName="PlatformUXTable" ref="A1:K7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -168,7 +169,7 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="FinanceTable" displayName="FinanceTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="SalaryTable" displayName="SalaryTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -187,7 +188,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="AttachmentsTable" displayName="AttachmentsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="FinanceTable" displayName="FinanceTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -206,7 +207,7 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CommunicationsTable" displayName="CommunicationsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="AttachmentsTable" displayName="AttachmentsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -225,7 +226,7 @@
 </file>
 
 <file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="PublicTrackingTable" displayName="PublicTrackingTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="CommunicationsTable" displayName="CommunicationsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -244,7 +245,26 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="DeploymentSmokeTable" displayName="DeploymentSmokeTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="PublicTrackingTable" displayName="PublicTrackingTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Test ID"/>
+    <x:tableColumn id="2" name="Priority"/>
+    <x:tableColumn id="3" name="Persona"/>
+    <x:tableColumn id="4" name="Tenant"/>
+    <x:tableColumn id="5" name="Preconditions"/>
+    <x:tableColumn id="6" name="Steps"/>
+    <x:tableColumn id="7" name="Expected Result"/>
+    <x:tableColumn id="8" name="Actual Result"/>
+    <x:tableColumn id="9" name="Status"/>
+    <x:tableColumn id="10" name="Automation"/>
+    <x:tableColumn id="11" name="Notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="17" name="DeploymentSmokeTable" displayName="DeploymentSmokeTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -339,7 +359,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -377,7 +397,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ProductionTable" displayName="ProductionTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ProductionTable" displayName="ProductionTable" ref="A1:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -396,7 +416,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="AttendanceTable" displayName="AttendanceTable" ref="A1:K13" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="WorkerContributionsTable" displayName="WorkerContributionsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -792,7 +812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf2c0d4684df4017"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78c06f89c1be4e6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -849,27 +869,27 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>UX-001</x:v>
+        <x:v>AT-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Any authorized user</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>A server mutation is available.</x:v>
+        <x:v>Active workers exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Click its submit CTA.</x:v>
+        <x:v>Mark daily attendance and save sheet.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>The CTA immediately shows a spinner and action-specific pending label and is disabled until completion.</x:v>
+        <x:v>One tenant-scoped attendance row per marked worker/date is saved.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -880,74 +900,74 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>UX-002</x:v>
+        <x:v>AT-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Any authorized user</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>A slow mutation is available.</x:v>
+        <x:v>Attendance data exists.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Submit, then attempt another CTA, navigation, dialog close, Escape, and rapid resubmit.</x:v>
+        <x:v>Open overview with 14-day range and worker filters.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Conflicting interaction is blocked, focused pending dialogs cannot close, and only one mutation is accepted.</x:v>
+        <x:v>Charts, regularity, and attention board reflect selected workers only.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual UI</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>UX-003</x:v>
+        <x:v>AT-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Any authorized user</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>An internal route link is available.</x:v>
+        <x:v>Tenant B worker ID known.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Click the link on desktop and mobile widths.</x:v>
+        <x:v>Submit attendance for Tenant B worker ID from Tenant A.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>A visible Opening page progress state appears and clears after navigation or the fail-safe timeout.</x:v>
+        <x:v>Action rejects worker ownership mismatch.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Manual UI</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
-    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="5" ht="66" hidden="0" customHeight="1">
       <x:c r="A5" s="6" t="str">
-        <x:v>UX-004</x:v>
+        <x:v>AT-004</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str">
         <x:v>Manager</x:v>
@@ -956,13 +976,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E5" s="6" t="str">
-        <x:v>A recoverable validation failure can be triggered in add-items or attendance import.</x:v>
+        <x:v>The supplied sample .xls report is available and some active worker profile names match exactly after normalization.</x:v>
       </x:c>
       <x:c r="F5" s="6" t="str">
-        <x:v>Submit invalid data.</x:v>
+        <x:v>Upload the report and preview it.</x:v>
       </x:c>
       <x:c r="G5" s="6" t="str">
-        <x:v>Error feedback is visible, the draft remains available, and retry succeeds without duplicate submission.</x:v>
+        <x:v>Preview writes nothing and shows report month, exact matches, unmatched/ambiguous workers, new/update rows, future dates, blank statuses, and unknown statuses.</x:v>
       </x:c>
       <x:c r="H5" s="6" t="str"/>
       <x:c r="I5" s="6" t="str">
@@ -971,74 +991,264 @@
       <x:c r="J5" s="6" t="str">
         <x:v>Manual + Automated</x:v>
       </x:c>
-      <x:c r="K5" s="6" t="str"/>
+      <x:c r="K5" s="6" t="str">
+        <x:v>Use docs_v2/sample_Attendance_Report.xls.</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A6" s="6" t="str">
-        <x:v>UX-005</x:v>
+        <x:v>AT-005</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str">
-        <x:v>Keyboard user</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D6" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
-        <x:v>Any shared dialog is available.</x:v>
+        <x:v>Preview contains matched and unmatched source workers.</x:v>
       </x:c>
       <x:c r="F6" s="6" t="str">
-        <x:v>Open it, tab through controls, press Shift+Tab at the first control, close it, and repeat during a pending save.</x:v>
+        <x:v>Confirm import.</x:v>
       </x:c>
       <x:c r="G6" s="6" t="str">
-        <x:v>Focus stays inside the modal, accessible name/description are exposed, focus returns to the trigger, and pending dialogs cannot close.</x:v>
+        <x:v>Only exact normalized active-worker matches are inserted or updated; no worker profiles are created and skipped names remain unchanged.</x:v>
       </x:c>
       <x:c r="H6" s="6" t="str"/>
       <x:c r="I6" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J6" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
-      </x:c>
-      <x:c r="K6" s="6" t="str"/>
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str">
+        <x:v>No fuzzy matching.</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A7" s="6" t="str">
-        <x:v>UX-006</x:v>
+        <x:v>AT-006</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str">
-        <x:v>Boutique user</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D7" s="6" t="str">
-        <x:v>Boutique-only tenant</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
-        <x:v>The user has a role that would otherwise permit Tasks.</x:v>
+        <x:v>Both tenants contain workers; a workbook name matches only Tenant B.</x:v>
       </x:c>
       <x:c r="F7" s="6" t="str">
-        <x:v>Open /tasks directly and attempt a Task server action.</x:v>
+        <x:v>Import while selected into Tenant A.</x:v>
       </x:c>
       <x:c r="G7" s="6" t="str">
-        <x:v>Both read and mutation paths reject access because Laundry is not enabled; Tasks remains hidden in navigation.</x:v>
+        <x:v>Tenant B worker and attendance rows are untouched; the source worker is skipped for Tenant A.</x:v>
       </x:c>
       <x:c r="H7" s="6" t="str"/>
       <x:c r="I7" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J7" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
+        <x:v>Database + Automated</x:v>
       </x:c>
       <x:c r="K7" s="6" t="str"/>
+    </x:row>
+    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>AT-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>A worker/date already has manual attendance and a note.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Preview and confirm a workbook containing that worker/date.</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Preview labels the row as an update; status/time/hours update atomically and the existing free-text note is preserved.</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str"/>
+    </x:row>
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>AT-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>A valid preview and idempotency key exist.</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Confirm twice or rapidly double-click confirmation.</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>The second request returns the stored receipt and creates no duplicate attendance or import receipt.</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>Database + Manual UI</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str"/>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>AT-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>A workbook contains a future date, blank status, unknown status, and duplicate normalized worker name.</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Preview and confirm.</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>Those rows/workers are explicitly reported and skipped; valid exact matches still import.</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str"/>
+      <x:c r="I10" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="str"/>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>AT-010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>A confirmed batch contains a tampered/invalid referenced row.</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Execute confirmation through the database contract.</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>The complete transaction rolls back and no partial attendance/import receipt remains.</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str"/>
+      <x:c r="I11" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str"/>
+    </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>AT-011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>A confirmed attendance import receipt exists.</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Attempt direct update and direct delete as service role, then delete its parent test tenant through approved cleanup.</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>Direct mutation is rejected as immutable; approved parent cascade cleanup remains possible.</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>Database</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str"/>
+    </x:row>
+    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>AT-012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>System</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>Adversarial .xlsx fixtures contain oversized expansion, unsafe ratios, local/central header mismatches, renamed extensions, or excessive entries/sheets/rows/columns/cells.</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Preview each fixture.</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>Every unsafe workbook is rejected before worksheet materialization via signature/header checks and hard-capped inflation; no receipt is written; valid .xls and .xlsx structures still reach format validation.</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str"/>
+      <x:c r="I13" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca95ffcf2e164898"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e37573a09f434a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1095,27 +1305,27 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>SA-001</x:v>
+        <x:v>UX-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Any authorized user</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Attendance and workers exist.</x:v>
+        <x:v>A server mutation is available.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create salary period and generate suggestions.</x:v>
+        <x:v>Click its submit CTA.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Suggestions derive from tenant workers, attendance, work logs, and ledger only.</x:v>
+        <x:v>The CTA immediately shows a spinner and action-specific pending label and is disabled until completion.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -1126,72 +1336,165 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+    <x:row r="3" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>SA-002</x:v>
+        <x:v>UX-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Any authorized user</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Existing active salary period.</x:v>
+        <x:v>A slow mutation is available.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Create overlapping salary period.</x:v>
+        <x:v>Submit, then attempt another CTA, navigation, dialog close, Escape, and rapid resubmit.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Action rejects overlap with clear message.</x:v>
+        <x:v>Conflicting interaction is blocked, focused pending dialogs cannot close, and only one mutation is accepted.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual UI</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>SA-003</x:v>
+        <x:v>UX-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Finance</x:v>
+        <x:v>Any authorized user</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Salary calculation exists.</x:v>
+        <x:v>An internal route link is available.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Finalize payable and record partial payment.</x:v>
+        <x:v>Click the link on desktop and mobile widths.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Final payable is preserved; salary_paid ledger entry appears in Finance rollup.</x:v>
+        <x:v>A visible Opening page progress state appears and clears after navigation or the fail-safe timeout.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
+        <x:v>Manual UI</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str"/>
+    </x:row>
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>UX-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>A recoverable validation failure can be triggered in add-items or attendance import.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Submit invalid data.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Error feedback is visible, the draft remains available, and retry succeeds without duplicate submission.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
         <x:v>Manual + Automated</x:v>
       </x:c>
-      <x:c r="K4" s="6" t="str"/>
+      <x:c r="K5" s="6" t="str"/>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>UX-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Keyboard user</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>Any shared dialog is available.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Open it, tab through controls, press Shift+Tab at the first control, close it, and repeat during a pending save.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Focus stays inside the modal, accessible name/description are exposed, focus returns to the trigger, and pending dialogs cannot close.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str"/>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>UX-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Boutique user</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Boutique-only tenant</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>The user has a role that would otherwise permit Tasks.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Open /tasks directly and attempt a Task server action.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>Both read and mutation paths reject access because Laundry is not enabled; Tasks remains hidden in navigation.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reacbea6ca5874ce7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97a49ee923db4d4f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1250,7 +1553,7 @@
     </x:row>
     <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>FI-001</x:v>
+        <x:v>SA-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
@@ -1262,13 +1565,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Expense category and payment mode exist.</x:v>
+        <x:v>Attendance and workers exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create expense.</x:v>
+        <x:v>Create salary period and generate suggestions.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Expense saves under selected tenant and appears in finance timeline.</x:v>
+        <x:v>Suggestions derive from tenant workers, attendance, work logs, and ledger only.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -1279,12 +1582,12 @@
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>FI-002</x:v>
+        <x:v>SA-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
         <x:v>Finance</x:v>
@@ -1293,58 +1596,58 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Customer/order payments and salary payments exist.</x:v>
+        <x:v>Existing active salary period.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open Finance overview.</x:v>
+        <x:v>Create overlapping salary period.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Cash in/out, salary expense rollup, dues, and P&amp;L are consistent.</x:v>
+        <x:v>Action rejects overlap with clear message.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>FI-003</x:v>
+        <x:v>SA-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Manager lacks finance permission.</x:v>
+        <x:v>Salary calculation exists.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Attempt finance write action.</x:v>
+        <x:v>Finalize payable and record partial payment.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Action is denied.</x:v>
+        <x:v>Final payable is preserved; salary_paid ledger entry appears in Finance rollup.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfab3561be0af45a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5198aeea1a6c49e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1403,101 +1706,101 @@
     </x:row>
     <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>AD-001</x:v>
+        <x:v>FI-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Customer exists.</x:v>
+        <x:v>Expense category and payment mode exist.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Upload JPG attachment on customer profile.</x:v>
+        <x:v>Create expense.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Attachment saves in private bucket and appears as thumbnail/gallery item.</x:v>
+        <x:v>Expense saves under selected tenant and appears in finance timeline.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
     <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>AD-002</x:v>
+        <x:v>FI-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Finance</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Tenant A and Tenant B</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Tenant B attachment ID known.</x:v>
+        <x:v>Customer/order payments and salary payments exist.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open download URL from Tenant A session.</x:v>
+        <x:v>Open Finance overview.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>No signed URL is issued.</x:v>
+        <x:v>Cash in/out, salary expense rollup, dues, and P&amp;L are consistent.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>AD-003</x:v>
+        <x:v>FI-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Customer-visible and internal attachments exist.</x:v>
+        <x:v>Manager lacks finance permission.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Open public tracking.</x:v>
+        <x:v>Attempt finance write action.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Internal/private attachments do not appear.</x:v>
+        <x:v>Action is denied.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e4aef33dc6a43fb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4abb5eb1be7b4174"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1556,101 +1859,101 @@
     </x:row>
     <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>CO-001</x:v>
+        <x:v>AD-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Owner/Admin</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Settings access.</x:v>
+        <x:v>Customer exists.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Create template with blocked variable such as {{worker_name}}.</x:v>
+        <x:v>Upload JPG attachment on customer profile.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Action rejects unsafe variable.</x:v>
+        <x:v>Attachment saves in private bucket and appears as thumbnail/gallery item.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
     <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>CO-002</x:v>
+        <x:v>AD-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P1</x:v>
+        <x:v>P0</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
         <x:v>Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
+        <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Order has customer phone/email.</x:v>
+        <x:v>Tenant B attachment ID known.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Queue manual tracking link dry-run.</x:v>
+        <x:v>Open download URL from Tenant A session.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Message queue and log are tenant-scoped and marked dry-run.</x:v>
+        <x:v>No signed URL is issued.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>CO-003</x:v>
+        <x:v>AD-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Owner/Admin</x:v>
+        <x:v>Public customer</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
+        <x:v>Public</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Communication channel settings open.</x:v>
+        <x:v>Customer-visible and internal attachments exist.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Attempt to set live mode.</x:v>
+        <x:v>Open public tracking.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Action rejects live sending in MVP slice.</x:v>
+        <x:v>Internal/private attachments do not appear.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4e0a11e67304145"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3c26c8f63a94da5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1707,105 +2010,103 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>PT-001</x:v>
+        <x:v>CO-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Valid tracking token exists.</x:v>
+        <x:v>Settings access.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Open /track/[token].</x:v>
+        <x:v>Create template with blocked variable such as {{worker_name}}.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>Page loads without Clerk and shows tenant branding, order dates, item names, and customer-safe statuses.</x:v>
+        <x:v>Action rejects unsafe variable.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J2" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
+        <x:v>Automated</x:v>
       </x:c>
       <x:c r="K2" s="6" t="str"/>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>PT-002</x:v>
+        <x:v>CO-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>P0</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Invalid/random token.</x:v>
+        <x:v>Order has customer phone/email.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open /track/random-token.</x:v>
+        <x:v>Queue manual tracking link dry-run.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Page returns not found.</x:v>
+        <x:v>Message queue and log are tenant-scoped and marked dry-run.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>PT-003</x:v>
+        <x:v>CO-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Public customer</x:v>
+        <x:v>Owner/Admin</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
-        <x:v>Public</x:v>
+        <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Order has measurements, workers, stage names, notes, salary, private attachments.</x:v>
+        <x:v>Communication channel settings open.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Open tracking token.</x:v>
+        <x:v>Attempt to set live mode.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>None of those internal fields appear in payload or UI.</x:v>
+        <x:v>Action rejects live sending in MVP slice.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
-      </x:c>
-      <x:c r="K4" s="6" t="str">
-        <x:v>Regression for 2026-06-04 hardening patch.</x:v>
-      </x:c>
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebb6f3d01ac242ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15938054ce914d62"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1862,6 +2163,161 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
+    <x:row r="2" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>PT-001</x:v>
+      </x:c>
+      <x:c r="B2" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C2" s="6" t="str">
+        <x:v>Public customer</x:v>
+      </x:c>
+      <x:c r="D2" s="6" t="str">
+        <x:v>Public</x:v>
+      </x:c>
+      <x:c r="E2" s="6" t="str">
+        <x:v>Valid tracking token exists.</x:v>
+      </x:c>
+      <x:c r="F2" s="6" t="str">
+        <x:v>Open /track/[token].</x:v>
+      </x:c>
+      <x:c r="G2" s="6" t="str">
+        <x:v>Page loads without Clerk and shows tenant branding, order dates, item names, and customer-safe statuses.</x:v>
+      </x:c>
+      <x:c r="H2" s="6" t="str"/>
+      <x:c r="I2" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J2" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K2" s="6" t="str"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>PT-002</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>Public customer</x:v>
+      </x:c>
+      <x:c r="D3" s="6" t="str">
+        <x:v>Public</x:v>
+      </x:c>
+      <x:c r="E3" s="6" t="str">
+        <x:v>Invalid/random token.</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="str">
+        <x:v>Open /track/random-token.</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="str">
+        <x:v>Page returns not found.</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="str"/>
+      <x:c r="I3" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J3" s="6" t="str">
+        <x:v>Automated</x:v>
+      </x:c>
+      <x:c r="K3" s="6" t="str"/>
+    </x:row>
+    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>PT-003</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>Public customer</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="str">
+        <x:v>Public</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Order has measurements, workers, stage names, notes, salary, private attachments.</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
+        <x:v>Open tracking token.</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>None of those internal fields appear in payload or UI.</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str"/>
+      <x:c r="I4" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J4" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K4" s="6" t="str">
+        <x:v>Regression for 2026-06-04 hardening patch.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de92db54f774992"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="15" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32.5" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="20" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="11.880000114440918" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16.25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="23.75" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="21" customHeight="1">
+      <x:c r="A1" s="4" t="str">
+        <x:v>Test ID</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="str">
+        <x:v>Priority</x:v>
+      </x:c>
+      <x:c r="C1" s="4" t="str">
+        <x:v>Persona</x:v>
+      </x:c>
+      <x:c r="D1" s="4" t="str">
+        <x:v>Tenant</x:v>
+      </x:c>
+      <x:c r="E1" s="4" t="str">
+        <x:v>Preconditions</x:v>
+      </x:c>
+      <x:c r="F1" s="4" t="str">
+        <x:v>Steps</x:v>
+      </x:c>
+      <x:c r="G1" s="4" t="str">
+        <x:v>Expected Result</x:v>
+      </x:c>
+      <x:c r="H1" s="4" t="str">
+        <x:v>Actual Result</x:v>
+      </x:c>
+      <x:c r="I1" s="4" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="J1" s="4" t="str">
+        <x:v>Automation</x:v>
+      </x:c>
+      <x:c r="K1" s="4" t="str">
+        <x:v>Notes</x:v>
+      </x:c>
+    </x:row>
     <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>DS-001</x:v>
@@ -1958,7 +2414,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcca074f367cf46c0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f440abbc5e94326"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2142,7 +2598,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0456c6f809314073"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5a60e6e90bd433b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2332,7 +2788,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a04a024ae7a4b83"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d455d4b5254ca8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2619,7 +3075,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c6bf608d1f74036"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43a93c5c1d554d92"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2772,7 +3228,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eb47fb2262b44fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bd9894e9bc14f69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3046,10 +3502,105 @@
       </x:c>
       <x:c r="K8" s="6" t="str"/>
     </x:row>
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>CF-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>Active stages and item types exist.</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Configure stage effort modes (assignment-only, units, hours, hybrid), then add compatible per-unit, per-hour, and percentage contribution rules; attempt an incompatible mode change.</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>Compatible rules save tenant-safely; the incompatible change is blocked with a recoverable message; active/completed stage snapshots are not rewritten.</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str">
+        <x:v>Contribution values are analytics-only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="66" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>CF-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>A stage has a saved effort mode.</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Edit its effort mode and save, then reopen the stage.</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>The dialog closes on success, visible feedback appears, and reopening shows the persisted mode rather than the prior default. A failed save keeps the editor and entered value open.</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str"/>
+      <x:c r="I10" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="str"/>
+    </x:row>
+    <x:row r="11" ht="79.19999694824219" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>CF-010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>Blazer stages support per-unit, per-hour, percentage, and no-rate cases.</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Save each rule, review the row summary, reopen one rule, and clear it with No monetary rule.</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>Each success exits edit mode and shows a plain-language saved summary; percentage explains the discounted pre-GST pool and allocation basis; clearing hides stale rate input and shows the unconfigured warning.</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str"/>
+      <x:c r="I11" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae819d272e534ccd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf91ec1c3e5041bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3268,7 +3819,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22b3cf844f3a416e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccec4ec49dc74cca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3418,10 +3969,394 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
+    <x:row r="5" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>PR-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>A ready stage maps to multiple workgroups and eligible active workers; one worker belongs to two eligible groups.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Open Start stage, add multiple workers, and choose the performed role for each row.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Every worker-role pair is explicit; duplicate pairs are rejected; the stage and all work logs start atomically.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str">
+        <x:v>The same worker may appear in different eligible roles, but not twice in the same role.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>PR-005</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C6" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E6" s="6" t="str">
+        <x:v>A unit-tracked stage has item quantity 2.</x:v>
+      </x:c>
+      <x:c r="F6" s="6" t="str">
+        <x:v>Credit 0.6 and 1.4 units to two workers, save, then complete; repeat with 0.25 and with a total other than 2.</x:v>
+      </x:c>
+      <x:c r="G6" s="6" t="str">
+        <x:v>Tenth-unit credits save; completion requires positive credit per worker and an exact 2-unit total; 0.25 and invalid totals roll back.</x:v>
+      </x:c>
+      <x:c r="H6" s="6" t="str"/>
+      <x:c r="I6" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J6" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K6" s="6" t="str"/>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>PR-006</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C7" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D7" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E7" s="6" t="str">
+        <x:v>An hour-tracked stage is ready for five eligible workers.</x:v>
+      </x:c>
+      <x:c r="F7" s="6" t="str">
+        <x:v>Assign five workers, add 1 hour to each using +10m/+1h controls, and complete after about one elapsed hour.</x:v>
+      </x:c>
+      <x:c r="G7" s="6" t="str">
+        <x:v>Total man-hours show 5h while elapsed stage/work-log time remains about 1h; time uses ten-minute increments.</x:v>
+      </x:c>
+      <x:c r="H7" s="6" t="str"/>
+      <x:c r="I7" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J7" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K7" s="6" t="str">
+        <x:v>Summed worker effort is intentionally independent of elapsed stage time.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>PR-007</x:v>
+      </x:c>
+      <x:c r="B8" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C8" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D8" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E8" s="6" t="str">
+        <x:v>A hybrid stage is ready.</x:v>
+      </x:c>
+      <x:c r="F8" s="6" t="str">
+        <x:v>Add multiple workers, enter both units and time, save partial effort, then complete with one worker missing either units or time.</x:v>
+      </x:c>
+      <x:c r="G8" s="6" t="str">
+        <x:v>Partial in-progress saves are allowed; completion requires positive units and time for every worker and exact total units.</x:v>
+      </x:c>
+      <x:c r="H8" s="6" t="str"/>
+      <x:c r="I8" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J8" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K8" s="6" t="str"/>
+    </x:row>
+    <x:row r="9" ht="66" hidden="0" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>PR-008</x:v>
+      </x:c>
+      <x:c r="B9" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C9" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D9" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E9" s="6" t="str">
+        <x:v>Item has a final after-discount, pre-GST value and item-type/stage rules exist.</x:v>
+      </x:c>
+      <x:c r="F9" s="6" t="str">
+        <x:v>Run per-unit, per-hour, percentage-by-units, and percentage-by-hours cases with multiple workers.</x:v>
+      </x:c>
+      <x:c r="G9" s="6" t="str">
+        <x:v>Fixed rules calculate per worker; percentage creates one pool from item final value and distributes it by credited effort with deterministic paise rounding; allocations sum exactly to the pool.</x:v>
+      </x:c>
+      <x:c r="H9" s="6" t="str"/>
+      <x:c r="I9" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J9" s="6" t="str">
+        <x:v>Automated + Manual</x:v>
+      </x:c>
+      <x:c r="K9" s="6" t="str">
+        <x:v>No per-worker duplication of a percentage pool.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>PR-009</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>A stage has no item-type contribution rule.</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Start, edit, and complete the stage.</x:v>
+      </x:c>
+      <x:c r="G10" s="6" t="str">
+        <x:v>A visible Rate not configured warning appears, production proceeds, and every calculated contribution is ₹0.</x:v>
+      </x:c>
+      <x:c r="H10" s="6" t="str"/>
+      <x:c r="I10" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J10" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K10" s="6" t="str">
+        <x:v>Configuration gaps never block production.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>PR-010</x:v>
+      </x:c>
+      <x:c r="B11" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C11" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D11" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E11" s="6" t="str">
+        <x:v>An in-progress stage has a worker with recorded units or time.</x:v>
+      </x:c>
+      <x:c r="F11" s="6" t="str">
+        <x:v>Remove that worker without a reason, then retry with a reason.</x:v>
+      </x:c>
+      <x:c r="G11" s="6" t="str">
+        <x:v>The first save is rejected atomically; the second soft-removes the active contribution and writes immutable old/new correction audit data.</x:v>
+      </x:c>
+      <x:c r="H11" s="6" t="str"/>
+      <x:c r="I11" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J11" s="6" t="str">
+        <x:v>Database + Manual</x:v>
+      </x:c>
+      <x:c r="K11" s="6" t="str">
+        <x:v>A worker with zero recorded effort may be removed without a reason.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="66" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>PR-011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>Manager and Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>A completed stage has snapshotted contributions.</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>As manager, attempt a direct completed correction; as owner/admin, correct worker effort with a reason.</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>Manager is denied server-side; owner/admin succeeds; original completion timestamps and elapsed duration remain unchanged; the audit reason is visible.</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>Database + Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str"/>
+    </x:row>
+    <x:row r="13" ht="66" hidden="0" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>PR-012</x:v>
+      </x:c>
+      <x:c r="B13" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C13" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D13" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E13" s="6" t="str">
+        <x:v>One stage is not started, one active, one completed; configuration is about to change.</x:v>
+      </x:c>
+      <x:c r="F13" s="6" t="str">
+        <x:v>Change the stage/rate configuration, then inspect all three and start the not-started stage.</x:v>
+      </x:c>
+      <x:c r="G13" s="6" t="str">
+        <x:v>Active/completed stages retain their snapshotted mode, rate, item value, and pool; only the newly started stage uses the new configuration; historical stages are not backfilled.</x:v>
+      </x:c>
+      <x:c r="H13" s="6" t="str"/>
+      <x:c r="I13" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J13" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K13" s="6" t="str"/>
+    </x:row>
+    <x:row r="14" ht="66" hidden="0" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>PR-013</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C14" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D14" s="6" t="str">
+        <x:v>Tenant A and Tenant B</x:v>
+      </x:c>
+      <x:c r="E14" s="6" t="str">
+        <x:v>Tenant B worker/workgroup/stage IDs are known and a valid Tenant A submission exists.</x:v>
+      </x:c>
+      <x:c r="F14" s="6" t="str">
+        <x:v>Submit foreign IDs, force an invalid row in a multi-worker save, rapidly submit twice, then replay the same idempotency key.</x:v>
+      </x:c>
+      <x:c r="G14" s="6" t="str">
+        <x:v>Foreign references and invalid batches roll back fully; duplicate submission creates one result; an exact replay returns the stored receipt; altered data with the same key is rejected.</x:v>
+      </x:c>
+      <x:c r="H14" s="6" t="str"/>
+      <x:c r="I14" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J14" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K14" s="6" t="str"/>
+    </x:row>
+    <x:row r="15" ht="52.79999923706055" hidden="0" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>PR-014</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="C15" s="6" t="str">
+        <x:v>Finance</x:v>
+      </x:c>
+      <x:c r="D15" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E15" s="6" t="str">
+        <x:v>Stage contributions exist alongside salary, order, GST, payment, expense, and ledger data.</x:v>
+      </x:c>
+      <x:c r="F15" s="6" t="str">
+        <x:v>Create and correct contributions, then compare all commercial and payroll records before and after.</x:v>
+      </x:c>
+      <x:c r="G15" s="6" t="str">
+        <x:v>Only contribution analytics/audit records change; salary, order totals, GST, payments, expenses, worker ledgers, and finance reports remain identical.</x:v>
+      </x:c>
+      <x:c r="H15" s="6" t="str"/>
+      <x:c r="I15" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J15" s="6" t="str">
+        <x:v>Database + Automated</x:v>
+      </x:c>
+      <x:c r="K15" s="6" t="str">
+        <x:v>Contribution reports remain analytics-only.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="66" hidden="0" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>PR-015</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C16" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D16" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E16" s="6" t="str">
+        <x:v>A unit/hybrid stage has item quantity 2 and two eligible workers.</x:v>
+      </x:c>
+      <x:c r="F16" s="6" t="str">
+        <x:v>Open Start stage, add a second worker, reallocate with -1/-0.1/+0.1/+1, and complete valid effort.</x:v>
+      </x:c>
+      <x:c r="G16" s="6" t="str">
+        <x:v>The first row starts at 2 units, the added row starts at zero, controls never exceed quantity or go below zero, and successful completion returns to the workflow view. Start/save remain open.</x:v>
+      </x:c>
+      <x:c r="H16" s="6" t="str"/>
+      <x:c r="I16" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J16" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K16" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R248fd2e4adae4e6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97f7ab3f62984ad6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3478,27 +4413,27 @@
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="2" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>AT-001</x:v>
+        <x:v>WC-001</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Owner/Admin or Manager</x:v>
       </x:c>
       <x:c r="D2" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E2" s="6" t="str">
-        <x:v>Active workers exist.</x:v>
+        <x:v>Completed contribution logs span multiple workers and weeks; one active log exists.</x:v>
       </x:c>
       <x:c r="F2" s="6" t="str">
-        <x:v>Mark daily attendance and save sheet.</x:v>
+        <x:v>As owner/admin open the dashboard report; as manager use Production &gt; Worker contributions. Switch between contribution value, units, man-hours, and completed stages.</x:v>
       </x:c>
       <x:c r="G2" s="6" t="str">
-        <x:v>One tenant-scoped attendance row per marked worker/date is saved.</x:v>
+        <x:v>Both approved roles can access the report without exposing unrelated dashboard modules; leaderboard and weekly trend use only completed logs, bucket by completion week, keep each metric separate, and show the correct tenant-scoped totals.</x:v>
       </x:c>
       <x:c r="H2" s="6" t="str"/>
       <x:c r="I2" s="6" t="str">
@@ -3507,357 +4442,76 @@
       <x:c r="J2" s="6" t="str">
         <x:v>Manual + Automated</x:v>
       </x:c>
-      <x:c r="K2" s="6" t="str"/>
-    </x:row>
-    <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="K2" s="6" t="str">
+        <x:v>No composite efficiency score.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="66" hidden="0" customHeight="1">
       <x:c r="A3" s="6" t="str">
-        <x:v>AT-002</x:v>
+        <x:v>WC-002</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Owner/Admin or Manager</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
-        <x:v>Attendance data exists.</x:v>
+        <x:v>Completed work includes configured and unconfigured contribution snapshots.</x:v>
       </x:c>
       <x:c r="F3" s="6" t="str">
-        <x:v>Open overview with 14-day range and worker filters.</x:v>
+        <x:v>Review report summary and a zero-value worker/stage.</x:v>
       </x:c>
       <x:c r="G3" s="6" t="str">
-        <x:v>Charts, regularity, and attention board reflect selected workers only.</x:v>
+        <x:v>Configuration coverage shows priced versus completed stages so a missing-rate zero is distinguishable; labels state analytics only and do not imply salary or revenue.</x:v>
       </x:c>
       <x:c r="H3" s="6" t="str"/>
       <x:c r="I3" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J3" s="6" t="str">
-        <x:v>Manual</x:v>
+        <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K3" s="6" t="str"/>
     </x:row>
-    <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="4" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A4" s="6" t="str">
-        <x:v>AT-003</x:v>
+        <x:v>WC-003</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str">
-        <x:v>Manager</x:v>
+        <x:v>Owner/Admin or Manager</x:v>
       </x:c>
       <x:c r="D4" s="6" t="str">
         <x:v>Tenant A and Tenant B</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
-        <x:v>Tenant B worker ID known.</x:v>
+        <x:v>Both tenants have completed contributions.</x:v>
       </x:c>
       <x:c r="F4" s="6" t="str">
-        <x:v>Submit attendance for Tenant B worker ID from Tenant A.</x:v>
+        <x:v>Open the report in each tenant using identical date ranges.</x:v>
       </x:c>
       <x:c r="G4" s="6" t="str">
-        <x:v>Action rejects worker ownership mismatch.</x:v>
+        <x:v>Every leaderboard, trend, and coverage value contains only the current tenant workers and logs.</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str"/>
       <x:c r="I4" s="6" t="str">
         <x:v>Not Run</x:v>
       </x:c>
       <x:c r="J4" s="6" t="str">
-        <x:v>Automated</x:v>
+        <x:v>Database + Automated</x:v>
       </x:c>
       <x:c r="K4" s="6" t="str"/>
-    </x:row>
-    <x:row r="5" ht="66" hidden="0" customHeight="1">
-      <x:c r="A5" s="6" t="str">
-        <x:v>AT-004</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C5" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D5" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E5" s="6" t="str">
-        <x:v>The supplied sample .xls report is available and some active worker profile names match exactly after normalization.</x:v>
-      </x:c>
-      <x:c r="F5" s="6" t="str">
-        <x:v>Upload the report and preview it.</x:v>
-      </x:c>
-      <x:c r="G5" s="6" t="str">
-        <x:v>Preview writes nothing and shows report month, exact matches, unmatched/ambiguous workers, new/update rows, future dates, blank statuses, and unknown statuses.</x:v>
-      </x:c>
-      <x:c r="H5" s="6" t="str"/>
-      <x:c r="I5" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J5" s="6" t="str">
-        <x:v>Manual + Automated</x:v>
-      </x:c>
-      <x:c r="K5" s="6" t="str">
-        <x:v>Use docs_v2/sample_Attendance_Report.xls.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="52.79999923706055" hidden="0" customHeight="1">
-      <x:c r="A6" s="6" t="str">
-        <x:v>AT-005</x:v>
-      </x:c>
-      <x:c r="B6" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C6" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D6" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E6" s="6" t="str">
-        <x:v>Preview contains matched and unmatched source workers.</x:v>
-      </x:c>
-      <x:c r="F6" s="6" t="str">
-        <x:v>Confirm import.</x:v>
-      </x:c>
-      <x:c r="G6" s="6" t="str">
-        <x:v>Only exact normalized active-worker matches are inserted or updated; no worker profiles are created and skipped names remain unchanged.</x:v>
-      </x:c>
-      <x:c r="H6" s="6" t="str"/>
-      <x:c r="I6" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J6" s="6" t="str">
-        <x:v>Database + Automated</x:v>
-      </x:c>
-      <x:c r="K6" s="6" t="str">
-        <x:v>No fuzzy matching.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A7" s="6" t="str">
-        <x:v>AT-006</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C7" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D7" s="6" t="str">
-        <x:v>Tenant A and Tenant B</x:v>
-      </x:c>
-      <x:c r="E7" s="6" t="str">
-        <x:v>Both tenants contain workers; a workbook name matches only Tenant B.</x:v>
-      </x:c>
-      <x:c r="F7" s="6" t="str">
-        <x:v>Import while selected into Tenant A.</x:v>
-      </x:c>
-      <x:c r="G7" s="6" t="str">
-        <x:v>Tenant B worker and attendance rows are untouched; the source worker is skipped for Tenant A.</x:v>
-      </x:c>
-      <x:c r="H7" s="6" t="str"/>
-      <x:c r="I7" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J7" s="6" t="str">
-        <x:v>Database + Automated</x:v>
-      </x:c>
-      <x:c r="K7" s="6" t="str"/>
-    </x:row>
-    <x:row r="8" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A8" s="6" t="str">
-        <x:v>AT-007</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C8" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D8" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E8" s="6" t="str">
-        <x:v>A worker/date already has manual attendance and a note.</x:v>
-      </x:c>
-      <x:c r="F8" s="6" t="str">
-        <x:v>Preview and confirm a workbook containing that worker/date.</x:v>
-      </x:c>
-      <x:c r="G8" s="6" t="str">
-        <x:v>Preview labels the row as an update; status/time/hours update atomically and the existing free-text note is preserved.</x:v>
-      </x:c>
-      <x:c r="H8" s="6" t="str"/>
-      <x:c r="I8" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J8" s="6" t="str">
-        <x:v>Database + Automated</x:v>
-      </x:c>
-      <x:c r="K8" s="6" t="str"/>
-    </x:row>
-    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A9" s="6" t="str">
-        <x:v>AT-008</x:v>
-      </x:c>
-      <x:c r="B9" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C9" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D9" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E9" s="6" t="str">
-        <x:v>A valid preview and idempotency key exist.</x:v>
-      </x:c>
-      <x:c r="F9" s="6" t="str">
-        <x:v>Confirm twice or rapidly double-click confirmation.</x:v>
-      </x:c>
-      <x:c r="G9" s="6" t="str">
-        <x:v>The second request returns the stored receipt and creates no duplicate attendance or import receipt.</x:v>
-      </x:c>
-      <x:c r="H9" s="6" t="str"/>
-      <x:c r="I9" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J9" s="6" t="str">
-        <x:v>Database + Manual UI</x:v>
-      </x:c>
-      <x:c r="K9" s="6" t="str"/>
-    </x:row>
-    <x:row r="10" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A10" s="6" t="str">
-        <x:v>AT-009</x:v>
-      </x:c>
-      <x:c r="B10" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C10" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D10" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E10" s="6" t="str">
-        <x:v>A workbook contains a future date, blank status, unknown status, and duplicate normalized worker name.</x:v>
-      </x:c>
-      <x:c r="F10" s="6" t="str">
-        <x:v>Preview and confirm.</x:v>
-      </x:c>
-      <x:c r="G10" s="6" t="str">
-        <x:v>Those rows/workers are explicitly reported and skipped; valid exact matches still import.</x:v>
-      </x:c>
-      <x:c r="H10" s="6" t="str"/>
-      <x:c r="I10" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J10" s="6" t="str">
-        <x:v>Automated</x:v>
-      </x:c>
-      <x:c r="K10" s="6" t="str"/>
-    </x:row>
-    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A11" s="6" t="str">
-        <x:v>AT-010</x:v>
-      </x:c>
-      <x:c r="B11" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C11" s="6" t="str">
-        <x:v>Manager</x:v>
-      </x:c>
-      <x:c r="D11" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E11" s="6" t="str">
-        <x:v>A confirmed batch contains a tampered/invalid referenced row.</x:v>
-      </x:c>
-      <x:c r="F11" s="6" t="str">
-        <x:v>Execute confirmation through the database contract.</x:v>
-      </x:c>
-      <x:c r="G11" s="6" t="str">
-        <x:v>The complete transaction rolls back and no partial attendance/import receipt remains.</x:v>
-      </x:c>
-      <x:c r="H11" s="6" t="str"/>
-      <x:c r="I11" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J11" s="6" t="str">
-        <x:v>Database</x:v>
-      </x:c>
-      <x:c r="K11" s="6" t="str"/>
-    </x:row>
-    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
-      <x:c r="A12" s="6" t="str">
-        <x:v>AT-011</x:v>
-      </x:c>
-      <x:c r="B12" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C12" s="6" t="str">
-        <x:v>System</x:v>
-      </x:c>
-      <x:c r="D12" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E12" s="6" t="str">
-        <x:v>A confirmed attendance import receipt exists.</x:v>
-      </x:c>
-      <x:c r="F12" s="6" t="str">
-        <x:v>Attempt direct update and direct delete as service role, then delete its parent test tenant through approved cleanup.</x:v>
-      </x:c>
-      <x:c r="G12" s="6" t="str">
-        <x:v>Direct mutation is rejected as immutable; approved parent cascade cleanup remains possible.</x:v>
-      </x:c>
-      <x:c r="H12" s="6" t="str"/>
-      <x:c r="I12" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J12" s="6" t="str">
-        <x:v>Database</x:v>
-      </x:c>
-      <x:c r="K12" s="6" t="str"/>
-    </x:row>
-    <x:row r="13" ht="79.19999694824219" hidden="0" customHeight="1">
-      <x:c r="A13" s="6" t="str">
-        <x:v>AT-012</x:v>
-      </x:c>
-      <x:c r="B13" s="6" t="str">
-        <x:v>P0</x:v>
-      </x:c>
-      <x:c r="C13" s="6" t="str">
-        <x:v>System</x:v>
-      </x:c>
-      <x:c r="D13" s="6" t="str">
-        <x:v>Phantom Threads</x:v>
-      </x:c>
-      <x:c r="E13" s="6" t="str">
-        <x:v>Adversarial .xlsx fixtures contain oversized expansion, unsafe ratios, local/central header mismatches, renamed extensions, or excessive entries/sheets/rows/columns/cells.</x:v>
-      </x:c>
-      <x:c r="F13" s="6" t="str">
-        <x:v>Preview each fixture.</x:v>
-      </x:c>
-      <x:c r="G13" s="6" t="str">
-        <x:v>Every unsafe workbook is rejected before worksheet materialization via signature/header checks and hard-capped inflation; no receipt is written; valid .xls and .xlsx structures still reach format validation.</x:v>
-      </x:c>
-      <x:c r="H13" s="6" t="str"/>
-      <x:c r="I13" s="6" t="str">
-        <x:v>Not Run</x:v>
-      </x:c>
-      <x:c r="J13" s="6" t="str">
-        <x:v>Automated</x:v>
-      </x:c>
-      <x:c r="K13" s="6" t="str"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R889b1657e31743e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9b9ef578b134274"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add garment icons and production filters
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R96ad21cb61d546eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R82c4f6f4e1f14435"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R9a62a31d409f4068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R20690d98c3624970"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R09ff56c615c347cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R6ade54b371b04a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R4d3c4cda2b0b4554"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="R9014ec8c76194146"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="R981c764b9baa48ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="R9129b09c68c54a42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="Rf595399044964d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="Rb7359c886cd84684"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="Rc313f18d089f4ac6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="Rae0df2c18cab4997"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R947e1a403ad0437b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R04cfb3c9642c4ec7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R7e8639b1f2684183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R1b9b9ff0eb544d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R2ea92411cadc4510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Rb1a4560ff9d54964"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R9bfdbdfa28d848f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R273f691d046e4cd2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="Raf732d15c7cb47a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R8b8096bb3d7c4bf1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="R11c85b9fde6540bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="Rbf246ac436b24dcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="Ref967d02c4174c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="Rca197618955c4643"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="Rc311a4e999a24420"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R7900348567254955"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="Rf5f33adb1e2a41be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R95c5967cdb784f3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R4e2f7100f8584444"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="Rf7d1c37dcbb24a68"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -397,7 +397,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ProductionTable" displayName="ProductionTable" ref="A1:K16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="ProductionTable" displayName="ProductionTable" ref="A1:K18" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -812,7 +812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78c06f89c1be4e6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b73f2f01f20469e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1248,7 +1248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9e37573a09f434a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a1dac057394d15"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,7 +1494,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97a49ee923db4d4f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75c9688401534116"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1647,7 +1647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5198aeea1a6c49e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d61c2996cd4e65"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1800,7 +1800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4abb5eb1be7b4174"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R626ccf716b1a49e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1953,7 +1953,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3c26c8f63a94da5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec564de6af54668"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2106,7 +2106,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15938054ce914d62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50c92b0d9632446f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2261,7 +2261,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1de92db54f774992"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd16d8e87c7f44f2f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2414,7 +2414,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f440abbc5e94326"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26e2a185fc046de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2598,7 +2598,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5a60e6e90bd433b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c534713c42647b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2788,7 +2788,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb3d455d4b5254ca8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cc0825cb6304f2d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3075,7 +3075,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43a93c5c1d554d92"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7ad4ca92c554fe1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3228,7 +3228,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bd9894e9bc14f69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3186fd0ca93147bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3600,7 +3600,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf91ec1c3e5041bf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R060357e4f78845e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3819,7 +3819,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccec4ec49dc74cca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bb0bb9128c34b6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4353,10 +4353,74 @@
       </x:c>
       <x:c r="K16" s="6" t="str"/>
     </x:row>
+    <x:row r="17" ht="66" hidden="0" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>PR-016</x:v>
+      </x:c>
+      <x:c r="B17" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C17" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D17" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E17" s="6" t="str">
+        <x:v>Two item types exist, one with an emoji and one without.</x:v>
+      </x:c>
+      <x:c r="F17" s="6" t="str">
+        <x:v>Create/edit the emoji, then inspect order creation, order detail, Production list/board, and workflow detail.</x:v>
+      </x:c>
+      <x:c r="G17" s="6" t="str">
+        <x:v>Exactly one emoji saves and appears internally; plain text or multiple emoji are rejected; the blank item type shows a neutral garment icon; public tracking does not expose the emoji.</x:v>
+      </x:c>
+      <x:c r="H17" s="6" t="str"/>
+      <x:c r="I17" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J17" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K17" s="6" t="str">
+        <x:v>Apply migration 20260809140000 first.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="66" hidden="0" customHeight="1">
+      <x:c r="A18" s="6" t="str">
+        <x:v>PR-017</x:v>
+      </x:c>
+      <x:c r="B18" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C18" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D18" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E18" s="6" t="str">
+        <x:v>Production contains several workflows and garment types.</x:v>
+      </x:c>
+      <x:c r="F18" s="6" t="str">
+        <x:v>Select two garment types and one workflow, then change search, queue, list/board view, and open/close a workflow pane.</x:v>
+      </x:c>
+      <x:c r="G18" s="6" t="str">
+        <x:v>Only matching tenant items appear and every active filter/view parameter is preserved; reset clears filters; foreign/unknown IDs never broaden results.</x:v>
+      </x:c>
+      <x:c r="H18" s="6" t="str"/>
+      <x:c r="I18" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J18" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K18" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97f7ab3f62984ad6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78353cea41d749ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4511,7 +4575,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9b9ef578b134274"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39c931e6a1c645b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: close successful action dialogs
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R1b9b9ff0eb544d84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R2ea92411cadc4510"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Rb1a4560ff9d54964"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R9bfdbdfa28d848f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R273f691d046e4cd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="Raf732d15c7cb47a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R8b8096bb3d7c4bf1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="R11c85b9fde6540bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="Rbf246ac436b24dcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="Ref967d02c4174c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="Rca197618955c4643"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="Rc311a4e999a24420"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R7900348567254955"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="Rf5f33adb1e2a41be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R95c5967cdb784f3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R4e2f7100f8584444"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="Rf7d1c37dcbb24a68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="Red885bc771dd4bd6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R13829d1dff974189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Re2995815a765471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R85becb137a594b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R8454ab2178fe4d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R946c839cd08143c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R0949ab8bed684b00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Re2760ada46d54312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="R0752b7c733834178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="Rd64ddf30448846ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="R23c01515bd4143d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R555326d265044a2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R1f907088d6e148a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R8bd346f6481c4f66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="Ra1c81749b7954fce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="Rbd82e9a511754068"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R3bcde59c86254510"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -207,7 +207,7 @@
 </file>
 
 <file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="AttachmentsTable" displayName="AttachmentsTable" ref="A1:K4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="AttachmentsTable" displayName="AttachmentsTable" ref="A1:K5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -359,7 +359,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="ConfigurationTable" displayName="ConfigurationTable" ref="A1:K12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="Test ID"/>
     <x:tableColumn id="2" name="Priority"/>
@@ -812,7 +812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b73f2f01f20469e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb193c42d73434fd2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1248,7 +1248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60a1dac057394d15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e330d4cd5df45ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,7 +1494,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R75c9688401534116"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4dfc36a010246c2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1647,7 +1647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64d61c2996cd4e65"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568aec1b75394440"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1800,7 +1800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R626ccf716b1a49e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77bf315d76dc4f8b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1950,10 +1950,41 @@
       </x:c>
       <x:c r="K4" s="6" t="str"/>
     </x:row>
+    <x:row r="5" ht="66" hidden="0" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>AD-004</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C5" s="6" t="str">
+        <x:v>Manager</x:v>
+      </x:c>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E5" s="6" t="str">
+        <x:v>An attachment-capable internal record is open.</x:v>
+      </x:c>
+      <x:c r="F5" s="6" t="str">
+        <x:v>Save one uploaded file and one external URL; repeat with an invalid submission.</x:v>
+      </x:c>
+      <x:c r="G5" s="6" t="str">
+        <x:v>Each success closes and resets the add dialog and the new card appears; invalid input stays open with data and error feedback; duplicate save is blocked while pending.</x:v>
+      </x:c>
+      <x:c r="H5" s="6" t="str"/>
+      <x:c r="I5" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J5" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K5" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdec564de6af54668"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re31cd06c1df2493f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2106,7 +2137,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50c92b0d9632446f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c86db89d0fa4421"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2261,7 +2292,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd16d8e87c7f44f2f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51832ff16ced4f0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2414,7 +2445,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb26e2a185fc046de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc85f4b6c7a74d5c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2598,7 +2629,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c534713c42647b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe452fa947d8498b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2788,7 +2819,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2cc0825cb6304f2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3cbde1954b647c3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3075,7 +3106,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7ad4ca92c554fe1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra804d41f80a54ec7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3228,7 +3259,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3186fd0ca93147bd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0ee40b75b74c73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3597,10 +3628,41 @@
       </x:c>
       <x:c r="K11" s="6" t="str"/>
     </x:row>
+    <x:row r="12" ht="66" hidden="0" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>CF-011</x:v>
+      </x:c>
+      <x:c r="B12" s="6" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="C12" s="6" t="str">
+        <x:v>Owner/Admin</x:v>
+      </x:c>
+      <x:c r="D12" s="6" t="str">
+        <x:v>Phantom Threads</x:v>
+      </x:c>
+      <x:c r="E12" s="6" t="str">
+        <x:v>Item type, stage, customer status, workgroup, payment mode, and expense category records exist.</x:v>
+      </x:c>
+      <x:c r="F12" s="6" t="str">
+        <x:v>Edit each record successfully, then force a validation error in one dialog.</x:v>
+      </x:c>
+      <x:c r="G12" s="6" t="str">
+        <x:v>Every successful dialog closes and shows confirmation; the pending dialog cannot close or double-submit; the failed dialog remains open with entered values and visible error feedback.</x:v>
+      </x:c>
+      <x:c r="H12" s="6" t="str"/>
+      <x:c r="I12" s="6" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="J12" s="6" t="str">
+        <x:v>Manual + Automated</x:v>
+      </x:c>
+      <x:c r="K12" s="6" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R060357e4f78845e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd53a59f0bfb439a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3819,7 +3881,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bb0bb9128c34b6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b254c067cd4cdd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4420,7 +4482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78353cea41d749ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1e3dbddf0d548d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4575,7 +4637,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39c931e6a1c645b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b0c81db9c53409c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: harden production filters and settings dialogs
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="Red885bc771dd4bd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R13829d1dff974189"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Re2995815a765471b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="R85becb137a594b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="R8454ab2178fe4d8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R946c839cd08143c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R0949ab8bed684b00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Re2760ada46d54312"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="R0752b7c733834178"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="Rd64ddf30448846ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="R23c01515bd4143d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R555326d265044a2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R1f907088d6e148a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R8bd346f6481c4f66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="Ra1c81749b7954fce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="Rbd82e9a511754068"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R3bcde59c86254510"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R949c9c8e092f4ebb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R6db3ef4f9adb4ccf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R7b3160e1deba47bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="Re782dfc99b9344f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rabf371424d784592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="Ra0ce7a1282484636"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R1fc9117c19fc4878"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="R0a66d6c07a30475a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="R9bdc553140184d40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="R7f3f181ead2c48d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="Rcecfce5d1a2a4bcf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R0d23f867829f4684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R8339f146217c44af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R2f3cbf4e477f48a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R5aa5a0d6e4f0483d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R853dbbeafaf14a0c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R345fa09f10344893"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -812,7 +812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb193c42d73434fd2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc64e26d7834b4bd3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1248,7 +1248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e330d4cd5df45ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11f4ea4b99394d68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,7 +1494,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4dfc36a010246c2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd55e8ac81a341d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1647,7 +1647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R568aec1b75394440"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd90b203ac6c84f85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1800,7 +1800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77bf315d76dc4f8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59e8f72d8de84d30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1984,7 +1984,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re31cd06c1df2493f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aa5c97a858b4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2137,7 +2137,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c86db89d0fa4421"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014b22a9687e4401"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2292,7 +2292,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R51832ff16ced4f0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f1267b588bb4e0f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2445,7 +2445,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdc85f4b6c7a74d5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R891a8e9ba3804319"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2629,7 +2629,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe452fa947d8498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50088ab708a3498b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2819,7 +2819,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3cbde1954b647c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbddb5bc34154899"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3106,7 +3106,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra804d41f80a54ec7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ec2b564f1454429"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3259,7 +3259,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe0ee40b75b74c73"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd97ae7fb6a644de6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3628,7 +3628,7 @@
       </x:c>
       <x:c r="K11" s="6" t="str"/>
     </x:row>
-    <x:row r="12" ht="66" hidden="0" customHeight="1">
+    <x:row r="12" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>CF-011</x:v>
       </x:c>
@@ -3642,13 +3642,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
-        <x:v>Item type, stage, customer status, workgroup, payment mode, and expense category records exist.</x:v>
+        <x:v>Master, workflow, measurement, user, location, team, and communication configuration records exist.</x:v>
       </x:c>
       <x:c r="F12" s="6" t="str">
-        <x:v>Edit each record successfully, then force a validation error in one dialog.</x:v>
+        <x:v>Edit each configuration record successfully, then force a validation error in one dialog.</x:v>
       </x:c>
       <x:c r="G12" s="6" t="str">
-        <x:v>Every successful dialog closes and shows confirmation; the pending dialog cannot close or double-submit; the failed dialog remains open with entered values and visible error feedback.</x:v>
+        <x:v>Every successful edit dialog closes and shows confirmation; pending dialogs cannot close or double-submit; failed dialogs remain open with entered values and visible error feedback; no nested forms are created.</x:v>
       </x:c>
       <x:c r="H12" s="6" t="str"/>
       <x:c r="I12" s="6" t="str">
@@ -3662,7 +3662,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdd53a59f0bfb439a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb42bab829e3f4c6f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3881,7 +3881,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7b254c067cd4cdd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90664a1fa6704e86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4448,7 +4448,7 @@
         <x:v>Apply migration 20260809140000 first.</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="66" hidden="0" customHeight="1">
+    <x:row r="18" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A18" s="6" t="str">
         <x:v>PR-017</x:v>
       </x:c>
@@ -4462,13 +4462,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
-        <x:v>Production contains several workflows and garment types.</x:v>
+        <x:v>Production contains more than 100 items across several workflows and garment types, including older matching items.</x:v>
       </x:c>
       <x:c r="F18" s="6" t="str">
-        <x:v>Select two garment types and one workflow, then change search, queue, list/board view, and open/close a workflow pane.</x:v>
+        <x:v>Select two garment types and one workflow; change search, queue, list/board view, and workflow pane; test both disclosures with keyboard and Escape.</x:v>
       </x:c>
       <x:c r="G18" s="6" t="str">
-        <x:v>Only matching tenant items appear and every active filter/view parameter is preserved; reset clears filters; foreign/unknown IDs never broaden results.</x:v>
+        <x:v>Predicates apply before the 100-row page limit so older matching items appear; all active URL state is preserved; reset clears filters; malformed/foreign IDs never broaden results; controls announce expanded state and Escape closes them.</x:v>
       </x:c>
       <x:c r="H18" s="6" t="str"/>
       <x:c r="I18" s="6" t="str">
@@ -4482,7 +4482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1e3dbddf0d548d1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra535d47d62d44d14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4637,7 +4637,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b0c81db9c53409c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf813c1ffca5b476a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add searchable item type icon picker
</commit_message>
<xml_diff>
--- a/docs/OS_PLUS_QA_Test_Matrix.xlsx
+++ b/docs/OS_PLUS_QA_Test_Matrix.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="R949c9c8e092f4ebb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R6db3ef4f9adb4ccf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="R7b3160e1deba47bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="Re782dfc99b9344f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rabf371424d784592"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="Ra0ce7a1282484636"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R1fc9117c19fc4878"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="R0a66d6c07a30475a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="R9bdc553140184d40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="R7f3f181ead2c48d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="Rcecfce5d1a2a4bcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R0d23f867829f4684"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R8339f146217c44af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R2f3cbf4e477f48a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="R5aa5a0d6e4f0483d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="R853dbbeafaf14a0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R345fa09f10344893"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Access" sheetId="1" r:id="Rda433e07ac304f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roles Permissions" sheetId="2" r:id="R5b3166cfb8654d5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tenant Isolation" sheetId="3" r:id="Rf5786b573b2d4f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="4" r:id="Ref99ef6dc20d489a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Measurements" sheetId="5" r:id="Rb4f72f9753d84c82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Configuration" sheetId="6" r:id="R1a736571103c425a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="7" r:id="R0f9bbdd89766400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production" sheetId="8" r:id="Rcff5f175c69845ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worker Contributions" sheetId="9" r:id="Rded4f65d623b4f99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance" sheetId="10" r:id="R58f4c2404dba4177"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform UX" sheetId="11" r:id="R483820667ae94283"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Salary" sheetId="12" r:id="R4e3937ce22ac43de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance" sheetId="13" r:id="R196ea2650d9c43f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attachments" sheetId="14" r:id="R73b74199c0884ea5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Communications" sheetId="15" r:id="Rcbbea6649fce437c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Public Tracking" sheetId="16" r:id="Rf501bac7686c40a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deployment Smoke" sheetId="17" r:id="R58e3027d51464f79"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -812,7 +812,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc64e26d7834b4bd3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad27cad41c6e415e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1248,7 +1248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11f4ea4b99394d68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfe559891e8e49c5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1494,7 +1494,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfd55e8ac81a341d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a9423a216654633"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1647,7 +1647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd90b203ac6c84f85"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R03e0ce6f94884bca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1800,7 +1800,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59e8f72d8de84d30"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6710e9e338f243e2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1984,7 +1984,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9aa5c97a858b4955"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70318252ea184232"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2137,7 +2137,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R014b22a9687e4401"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f72d013c5c742c0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2292,7 +2292,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f1267b588bb4e0f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a2d81de595426d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2445,7 +2445,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R891a8e9ba3804319"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a15f33e035543bf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2629,7 +2629,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50088ab708a3498b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f5b06120f4d4a04"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2819,7 +2819,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdbddb5bc34154899"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62cf54a600bb411a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3106,7 +3106,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ec2b564f1454429"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43412d8656404228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3259,7 +3259,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd97ae7fb6a644de6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R969d71460bb4493a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3662,7 +3662,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb42bab829e3f4c6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9e623bcefc4389"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3881,7 +3881,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90664a1fa6704e86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cb1abe9b6f342d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4415,7 +4415,7 @@
       </x:c>
       <x:c r="K16" s="6" t="str"/>
     </x:row>
-    <x:row r="17" ht="66" hidden="0" customHeight="1">
+    <x:row r="17" ht="118.80000305175781" hidden="0" customHeight="1">
       <x:c r="A17" s="6" t="str">
         <x:v>PR-016</x:v>
       </x:c>
@@ -4429,13 +4429,13 @@
         <x:v>Phantom Threads</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
-        <x:v>Two item types exist, one with an emoji and one without.</x:v>
+        <x:v>Both item-type icon migrations are applied and create/edit item-type forms are available.</x:v>
       </x:c>
       <x:c r="F17" s="6" t="str">
-        <x:v>Create/edit the emoji, then inspect order creation, order detail, Production list/board, and workflow detail.</x:v>
+        <x:v>Enter item names from boutique, laundry, food, and repair domains; open Suggested, search Emoji and Icons, change skin tone and icon color, reopen recent choices, then choose Default. Inspect order creation, order detail, Production list/board, and workflow detail at 320 px and desktop widths.</x:v>
       </x:c>
       <x:c r="G17" s="6" t="str">
-        <x:v>Exactly one emoji saves and appears internally; plain text or multiple emoji are rejected; the blank item type shows a neutral garment icon; public tracking does not expose the emoji.</x:v>
+        <x:v>Suggested choices respond to the name and retain recent local choices; all library tabs are keyboard-operable with named 44 px targets; emoji/skin tone and Lucide name/color save and reopen; invalid or mixed values fail server validation without losing input; Default is neutral; public tracking exposes no icon; normal pages do not load the picker catalogue.</x:v>
       </x:c>
       <x:c r="H17" s="6" t="str"/>
       <x:c r="I17" s="6" t="str">
@@ -4445,7 +4445,7 @@
         <x:v>Manual + Automated</x:v>
       </x:c>
       <x:c r="K17" s="6" t="str">
-        <x:v>Apply migration 20260809140000 first.</x:v>
+        <x:v>Apply migrations 20260809140000 and 20260809150000 first; verify /emoji-data/en/data.json and messages.json return 200.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="79.19999694824219" hidden="0" customHeight="1">
@@ -4482,7 +4482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra535d47d62d44d14"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d8755ad1983420b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4637,7 +4637,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf813c1ffca5b476a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6c6c7466c6a4b51"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>